<commit_message>
Fix ZA album: Add ZA to AlbumWinner enum and correct image URLs
- Added 'ZA' to album_id enum in AlbumWinner model to allow winner registration
- Fixed all Braze image URLs in createZAAlbumExcel.js (corrected Castle Lager 10pts URL)
- Regenerated AlbumStockZA.xlsx with correct Braze CDN URLs
- This fixes the issue where winners couldn't be registered for South Africa album

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Files/AlbumStockZA.xlsx
+++ b/Files/AlbumStockZA.xlsx
@@ -442,7 +442,7 @@
         <v>Castle Lager 10pts</v>
       </c>
       <c r="D2" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_10pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962677897580083c6b269/original.jpg?1780048486</v>
       </c>
       <c r="E2">
         <v>10</v>
@@ -465,7 +465,7 @@
         <v>Castle Lager 20pts</v>
       </c>
       <c r="D3" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_20pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196267eef5080083fee44d/original.jpg?1780048486</v>
       </c>
       <c r="E3">
         <v>20</v>
@@ -488,7 +488,7 @@
         <v>Castle Lager 30pts</v>
       </c>
       <c r="D4" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_30pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962685f9c650081a0c30d/original.jpg?1780048487</v>
       </c>
       <c r="E4">
         <v>30</v>
@@ -511,7 +511,7 @@
         <v>Castle Lager 40pts</v>
       </c>
       <c r="D5" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_40pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962687a647b00835879fa/original.jpg?1780048487</v>
       </c>
       <c r="E5">
         <v>40</v>
@@ -534,7 +534,7 @@
         <v>Castle Lager 50pts</v>
       </c>
       <c r="D6" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_50pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196268b9a59f00831e71fd/original.jpg?1780048487</v>
       </c>
       <c r="E6">
         <v>50</v>
@@ -557,7 +557,7 @@
         <v>Castle Lager 75pts</v>
       </c>
       <c r="D7" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_75pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962671e6c75008373a37e/original.jpg?1780048487</v>
       </c>
       <c r="E7">
         <v>75</v>
@@ -580,7 +580,7 @@
         <v>Castle Lager 100pts</v>
       </c>
       <c r="D8" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_100pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962696437bc0083fcea60/original.jpg?1780048488</v>
       </c>
       <c r="E8">
         <v>100</v>
@@ -603,7 +603,7 @@
         <v>Castle Lager 200pts</v>
       </c>
       <c r="D9" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_200pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962690879ed00816dd24c/original.jpg?1780048488</v>
       </c>
       <c r="E9">
         <v>200</v>
@@ -626,7 +626,7 @@
         <v>Castle Lager 250pts</v>
       </c>
       <c r="D10" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_250pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196269988a840085f17b36/original.png?1780048488</v>
       </c>
       <c r="E10">
         <v>250</v>
@@ -649,7 +649,7 @@
         <v>Castle Lager 500pts</v>
       </c>
       <c r="D11" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_500pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962690879ed009c6db7bf/original.jpg?1780048489</v>
       </c>
       <c r="E11">
         <v>500</v>
@@ -672,7 +672,7 @@
         <v>Castle Lager No Prize 1</v>
       </c>
       <c r="D12" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_NoPrize1.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19626a50ef120083d28611/original.png?1780048489</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -695,7 +695,7 @@
         <v>Castle Lager No Prize 2</v>
       </c>
       <c r="D13" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CastleLager_NoPrize2.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19626a50ef120083d28611/original.png?1780048489</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -718,7 +718,7 @@
         <v>Flying Fish 10pts</v>
       </c>
       <c r="D14" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_10pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1964021732ec0086542fda/original.jpeg?1780048897</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -741,7 +741,7 @@
         <v>Flying Fish 20pts</v>
       </c>
       <c r="D15" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_20pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196402d483e50083b2d8ba/original.jpeg?1780048897</v>
       </c>
       <c r="E15">
         <v>20</v>
@@ -764,7 +764,7 @@
         <v>Flying Fish 30pts</v>
       </c>
       <c r="D16" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_30pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196402cfcd520081cdabbf/original.jpeg?1780048898</v>
       </c>
       <c r="E16">
         <v>30</v>
@@ -787,7 +787,7 @@
         <v>Flying Fish 40pts</v>
       </c>
       <c r="D17" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_40pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196403d886f000833b1735/original.jpeg?1780048899</v>
       </c>
       <c r="E17">
         <v>40</v>
@@ -810,7 +810,7 @@
         <v>Flying Fish 50pts</v>
       </c>
       <c r="D18" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_50pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19640427d35600832d47e7/original.jpeg?1780048899</v>
       </c>
       <c r="E18">
         <v>50</v>
@@ -833,7 +833,7 @@
         <v>Flying Fish 75pts</v>
       </c>
       <c r="D19" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_75pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1964028bba4d0083d37448/original.jpeg?1780048897</v>
       </c>
       <c r="E19">
         <v>75</v>
@@ -856,7 +856,7 @@
         <v>Flying Fish 100pts</v>
       </c>
       <c r="D20" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_100pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196403eedda8008361942b/original.jpeg?1780048899</v>
       </c>
       <c r="E20">
         <v>100</v>
@@ -879,7 +879,7 @@
         <v>Flying Fish 200pts</v>
       </c>
       <c r="D21" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_200pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196403628289008173a0e5/original.jpeg?1780048899</v>
       </c>
       <c r="E21">
         <v>200</v>
@@ -902,7 +902,7 @@
         <v>Flying Fish 250pts</v>
       </c>
       <c r="D22" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_250pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19640398b6440081ecb4ea/original.jpeg?1780048899</v>
       </c>
       <c r="E22">
         <v>250</v>
@@ -925,7 +925,7 @@
         <v>Flying Fish 500pts</v>
       </c>
       <c r="D23" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_500pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1964035f05210083976b21/original.jpeg?1780048899</v>
       </c>
       <c r="E23">
         <v>500</v>
@@ -948,7 +948,7 @@
         <v>Flying Fish No Prize 1</v>
       </c>
       <c r="D24" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_NoPrize1.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19640527fe98008194252c/original.png?1780048900</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -971,7 +971,7 @@
         <v>Flying Fish No Prize 2</v>
       </c>
       <c r="D25" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_FlyingFish_NoPrize2.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19640527fe98008194252c/original.png?1780048900</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -994,7 +994,7 @@
         <v>Carling Black Label 10pts</v>
       </c>
       <c r="D26" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_10pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f65cb0c7c0081c8fffd/original.jpeg?1780047716</v>
       </c>
       <c r="E26">
         <v>10</v>
@@ -1017,7 +1017,7 @@
         <v>Carling Black Label 20pts</v>
       </c>
       <c r="D27" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_20pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1961a834a9150083909f7c/original.png?1780048295</v>
       </c>
       <c r="E27">
         <v>20</v>
@@ -1040,7 +1040,7 @@
         <v>Carling Black Label 30pts</v>
       </c>
       <c r="D28" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_30pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1961a86adf0a008168e81d/original.png?1780048295</v>
       </c>
       <c r="E28">
         <v>30</v>
@@ -1063,7 +1063,7 @@
         <v>Carling Black Label 40pts</v>
       </c>
       <c r="D29" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_40pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f647138800083095d1c/original.jpg?1780047716</v>
       </c>
       <c r="E29">
         <v>40</v>
@@ -1086,7 +1086,7 @@
         <v>Carling Black Label 50pts</v>
       </c>
       <c r="D30" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_50pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f647b6d450083b1f883/original.jpg?1780047716</v>
       </c>
       <c r="E30">
         <v>50</v>
@@ -1109,7 +1109,7 @@
         <v>Carling Black Label 75pts</v>
       </c>
       <c r="D31" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_75pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f66997c7f00833d42a3/original.jpg?1780047718</v>
       </c>
       <c r="E31">
         <v>75</v>
@@ -1132,7 +1132,7 @@
         <v>Carling Black Label 100pts</v>
       </c>
       <c r="D32" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_100pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f67ad718f0081b0d45c/original.jpeg?1780047718</v>
       </c>
       <c r="E32">
         <v>100</v>
@@ -1155,7 +1155,7 @@
         <v>Carling Black Label 200pts</v>
       </c>
       <c r="D33" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_200pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f689a4a48008539f51e/original.jpeg?1780047719</v>
       </c>
       <c r="E33">
         <v>200</v>
@@ -1178,7 +1178,7 @@
         <v>Carling Black Label 250pts</v>
       </c>
       <c r="D34" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_250pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f6799ce2f008138bc9a/original.jpg?1780047718</v>
       </c>
       <c r="E34">
         <v>250</v>
@@ -1201,7 +1201,7 @@
         <v>Carling Black Label 500pts</v>
       </c>
       <c r="D35" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_500pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f670ba3cc0083b53689/original.jpg?1780047718</v>
       </c>
       <c r="E35">
         <v>500</v>
@@ -1224,7 +1224,7 @@
         <v>Carling Black Label No Prize 1</v>
       </c>
       <c r="D36" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_NoPrize1.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1961ab8712a30083578501/original.png?1780048298</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -1247,7 +1247,7 @@
         <v>Carling Black Label No Prize 2</v>
       </c>
       <c r="D37" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_CarlingBlackLabel_NoPrize2.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1961ab8712a30083578501/original.png?1780048298</v>
       </c>
       <c r="E37">
         <v>0</v>
@@ -1270,7 +1270,7 @@
         <v>All Brands 10pts</v>
       </c>
       <c r="D38" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_10pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f65cb0c7c0081c8fffd/original.jpeg?1780047716</v>
       </c>
       <c r="E38">
         <v>10</v>
@@ -1293,7 +1293,7 @@
         <v>All Brands 20pts</v>
       </c>
       <c r="D39" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_20pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196267eef5080083fee44d/original.jpg?1780048486</v>
       </c>
       <c r="E39">
         <v>20</v>
@@ -1316,7 +1316,7 @@
         <v>All Brands 30pts</v>
       </c>
       <c r="D40" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_30pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196402cfcd520081cdabbf/original.jpeg?1780048898</v>
       </c>
       <c r="E40">
         <v>30</v>
@@ -1339,7 +1339,7 @@
         <v>All Brands 40pts</v>
       </c>
       <c r="D41" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_40pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f647138800083095d1c/original.jpg?1780047716</v>
       </c>
       <c r="E41">
         <v>40</v>
@@ -1362,7 +1362,7 @@
         <v>All Brands 50pts</v>
       </c>
       <c r="D42" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_50pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196268b9a59f00831e71fd/original.jpg?1780048487</v>
       </c>
       <c r="E42">
         <v>50</v>
@@ -1385,7 +1385,7 @@
         <v>All Brands 75pts</v>
       </c>
       <c r="D43" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_75pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962671e6c75008373a37e/original.jpg?1780048487</v>
       </c>
       <c r="E43">
         <v>75</v>
@@ -1408,7 +1408,7 @@
         <v>All Brands 100pts</v>
       </c>
       <c r="D44" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_100pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196403eedda8008361942b/original.jpeg?1780048899</v>
       </c>
       <c r="E44">
         <v>100</v>
@@ -1431,7 +1431,7 @@
         <v>All Brands 200pts</v>
       </c>
       <c r="D45" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_200pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1962690879ed00816dd24c/original.jpg?1780048488</v>
       </c>
       <c r="E45">
         <v>200</v>
@@ -1454,7 +1454,7 @@
         <v>All Brands 250pts</v>
       </c>
       <c r="D46" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_250pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a196269988a840085f17b36/original.png?1780048488</v>
       </c>
       <c r="E46">
         <v>250</v>
@@ -1477,7 +1477,7 @@
         <v>All Brands 500pts</v>
       </c>
       <c r="D47" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_500pts.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a195f670ba3cc0083b53689/original.jpg?1780047718</v>
       </c>
       <c r="E47">
         <v>500</v>
@@ -1500,7 +1500,7 @@
         <v>All Brands No Prize 1</v>
       </c>
       <c r="D48" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_NoPrize1.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a1961ab8712a30083578501/original.png?1780048298</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -1523,7 +1523,7 @@
         <v>All Brands No Prize 2</v>
       </c>
       <c r="D49" t="str">
-        <v>https://mysiterobert.s3.us-east-1.amazonaws.com/BEES_2026/Album2026/ZA/ZA_AllBrands_NoPrize2.png</v>
+        <v>https://braze-images.com/appboy/communication/assets/image_assets/images/6a19626a50ef120083d28611/original.png?1780048489</v>
       </c>
       <c r="E49">
         <v>0</v>

</xml_diff>